<commit_message>
added logo and some moe info on app
</commit_message>
<xml_diff>
--- a/SHA values and test data.xlsx
+++ b/SHA values and test data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\paarl\source\repos\Sha256Gui\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FA21F6A7-127D-448F-B859-24305BBE5EBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2AE0072-A1F4-4E62-AF2A-956F34A9761A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{2E73F5BF-DE38-4323-B1CD-402605A793B9}"/>
   </bookViews>
@@ -140,9 +140,6 @@
     <t>irJ/0YrdJobuobMVc/uUP/zrO3HKUkfc1joRge1siAKtumpN2HvFN2H41VX5QAclZzbkerdoAabGOykIh4hxGsAtrWH3AEUetQYKFKML/pexmoa/XKAUVtus6VXzwC8UfgFaOuf9PrvVwlw7h4XPri0HTD6zlb5lp/ZtmWUObZsCxq4PiwGhT/7wVFChtqfPZ/urRWSkV+cf/Ca5aO7qdNSgewB5kgbFcEWAah7uxOFSVuSTycfAHd1sEqf7FA6+xGf9LDy/F300M5eTlnHhdZ8a8aGYbiDdO7jtoueGAFLsTiCCsph64p8tqkZFtiP0jXQUJW0/Gkg26mQgOeoT16visroiwX8gLC7FGaLXRrZ7mCkPfoszXQU9+55X0t1J8dOZoVy4Y1V48xv53pRxyfdj60AakPfWzVwMwNr0KG8MKM9dR6gPm7B0f7dKU+MsZ06cYU+5w14SCDQGpr8H2kG262ON9zd0A83LfSGdyVX7d1bFYb8dFJHB3RENXoXS8iGv+XSmUxwsCk4KCq02Ke7lKo9DQ5g5Fi8Fcr0FSMSG/RBMrhQRg9JOSfgCfdHuVpnpAr4rRKrj8GaYPOCpaDDt4BpyR/DO99HSoTewAYVsF0/RxKg/Gzn0FubOKAeVgBaQfB4pkVuKpa6fZWH1U6xfZeEeyJ2NP/ZcTQkieweQfSjSsxWWH1avm6zU3HeovzRybzVme2Y0GN+TTJDdBsqj8gW7iKqDqMYRgPV3MJZPpwwUrPD7OAdyug6oGH7Vmrnv62CHiqFl+TCyYBw0dRqs9s3nQTLgVIXCCLBnLvcOdmi4aoWs+nSq3AJGVnwKrPdmGLLh4FsOqPoYIJzzB2yRmcuNOxV9JTvQK/9C0ldyeLDbkvbVHZISQiZNBZsFzjs/IjDhKd64HHdGrDgBmF4o3zYDXWb64HFvB7+QODp+jwWGyiTFtYAWeIAC1l5xhXZiMozfMi4kqH0/KjCsYcv8yuiQ36Rw6SkXu1QHjYn6oOXoxhDdJr/YVCG3pVyEK47C1n6ps6F0tJpnlRrQSE5T5mz0QZgtpQTZ5a99H/bmzE8hufWjvfPvEy8AXxYm8CM/1L11PhdbxF8ohCi+btC9ga53Fi1RbcCqZGCyGVX2GL/SAPOny6whGtubdI97SHtgZWvFBayyk/dXQ+Go/g7KzqZ4LuH+euTbWCSBAV/Mwb9LMOSQ6V/gmXOGhAHqTmEKxw91N46bOq+PSo3R/Mz64chCOmBsp+5Tt5MvkGEwcvT8Zo3KRUgFP0M9k376c3X8mCqCswdpCSe6yxBBoyaKFs8VfqDorbZsn3sUD0PmhoaQ4R9zGqCr9EGJeWd/K2aAlDnZws0dzBSYNP1w6mdosITz8Rv+Fxr1pzxkbgMm3ssgdZucktL5Mkw2c7J/iSE82yMHBQIA9yvGSMmP/cKYUdYhU8q6cgCyNAQd6hBjvapKmes8psnpim8zf1E4+MTV6hYQaEZP+kvjbfbaVHTHVIaHI7lSlTwDb1xLHz5jXMSx5oM8awTmAE1RJp6g4Wjk6QuIF8OXosbcAzioZ7lq9vkW+MiTQD6t5hYx+NYKgLSnmWxMxwltLO847dtIiHkrMo9ZEtt/RpvtoSkWhtGTmAmxWnbkFKU+swZEDMgIlJfc+AI8H06NePqCAN1887vnPvN2zNRA4F/VdiIHq3EdLHtFLJVSoLsRgHqcDZYGjCgcIQJiLVgdr7r2LS8eu3Nz/alU7yLi7ZSRGgT0EdGSSGrm2PBA4XtYDtaGUCDSaiBdTmP26PowjM4VY0q3uLUp0H1uKtc5pxplmO88wco75mD3ADB2NnC0/uS/p+Szz+b6aYJamzwEIH/TOd0FblQ90txRtRrgNZ0UVNpw1Nuf7Ii7EQVBh3M1AhqRo5tZoJBvsfwCkUPqPaoCuB4tNsyl+FgUpx+um1MHE6u4Izf7z2QZ+vXr2twGnmq5VCaxC59wLR40wMLkEbTOK5oMcjFmmmQi2srC7cvZm6d5iX+GbtRr1AF7LH0UYczHNfI0zvUl86Ya/IlOXUFdnk8JzKZBRQj+aHS/LBP+k/CpJcrfKs2Rt3IR2s8fAlyovOiJga0niAvfHNMnVMYb1msu+Iy08LUxZY/qM9WAKo1knkl+H8dOptsRBKehH3CRq53Vl4Op2QOP9B6sgDW5j9oMWfMGEKoNPLRGVlMxF/agkDHZa8UHeEfxpvvQvk0OZe6y7IuHJMOjuCbFpbUUzKd+mbjeKcnp3gZXunRIKHc+Enp1R9/VDixoC7wenWRksAZBpAH43RX47OeTfRNQ2TFc2u2UmeYeVZdUB+VtWZvHPB+2uOQMnR6SbMMggfOnArQLvp3drV6MK3YgvaQJY2kEluFKZkFnRcdzaqBlD1vWJuOA+/XBxf6M9oGnUZrWwOKukA+2bfM4SB4D4CNgvHMAtqk4WlAaKT50DqgKU838w3B2HuICadcv132hLyyHV+o/gRt5gYCa4ePsqqXPtL2Ez0FtE1VfVF2BnHDUeFZly6HPlSVqdzDfPqE/aYQSKMpQE9s27mvFstg1Gq1vybO7koRjVlpW448eUPCbxpsfGnuKlxueU1+kyixQcK7ALMpbPqFcSvUoH1qy0XZAGAEZ+sJiTYbKNQbhSeLtGtVhwHwrBp9p+JvZhY0xl58/eSjsz/j06DVawwoiO99uQzZt3PimGXVbYt1Xz/WlUbiF4Q==</t>
   </si>
   <si>
-    <t>Take all info in table above , including th header.  Get SHA256 of A, then use that SHA value as a key for AES encryption you get:</t>
-  </si>
-  <si>
     <t>Cryptext:</t>
   </si>
   <si>
@@ -150,16 +147,42 @@
   </si>
   <si>
     <t>Use the OpenCrypTool.exe (SHa256GUI repositry</t>
+  </si>
+  <si>
+    <t>Take all info in table above , including the headers.  Get SHA256 of A (A is the secret I used here), then use that SHA value as a key for AES encryption you get:</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -185,12 +208,21 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -551,13 +583,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F7AB10E-06D4-4937-8761-61927B0A545B}">
-  <dimension ref="A1:D29"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.140625" style="1" customWidth="1"/>
     <col min="2" max="2" width="67.28515625" style="2" customWidth="1"/>
     <col min="3" max="3" width="85" style="2" customWidth="1"/>
-    <col min="4" max="16384" width="9.140625" style="1"/>
+    <col min="4" max="4" width="82.85546875" style="1" customWidth="1"/>
+    <col min="5" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
@@ -679,18 +712,18 @@
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B13" s="2" t="s">
+      <c r="B13" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="B14" s="5" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="B14" s="2" t="s">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B15" s="3" t="s">
         <v>33</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B15" s="2" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
@@ -698,128 +731,139 @@
         <v>32</v>
       </c>
     </row>
-    <row r="18" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B18" s="2" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="19" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B18" s="3" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="19" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B19" s="2" t="s">
         <v>1</v>
       </c>
       <c r="C19" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D19" s="1" t="s">
+      <c r="D19" s="2" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="20" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="E19" s="2"/>
+    </row>
+    <row r="20" spans="2:5" ht="30" x14ac:dyDescent="0.25">
       <c r="C20" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="D20" s="1" t="s">
+      <c r="D20" s="2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="21" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="E20" s="2"/>
+    </row>
+    <row r="21" spans="2:5" ht="30" x14ac:dyDescent="0.25">
       <c r="B21" s="2" t="s">
         <v>0</v>
       </c>
       <c r="C21" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="D21" s="1" t="s">
+      <c r="D21" s="2" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="22" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="E21" s="2"/>
+    </row>
+    <row r="22" spans="2:5" ht="30" x14ac:dyDescent="0.25">
       <c r="B22" s="2" t="s">
         <v>9</v>
       </c>
       <c r="C22" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="D22" s="1" t="s">
+      <c r="D22" s="2" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="23" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="E22" s="2"/>
+    </row>
+    <row r="23" spans="2:5" ht="30" x14ac:dyDescent="0.25">
       <c r="B23" s="2" t="s">
         <v>11</v>
       </c>
       <c r="C23" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="D23" s="1" t="s">
+      <c r="D23" s="2" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="24" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="E23" s="2"/>
+    </row>
+    <row r="24" spans="2:5" ht="30" x14ac:dyDescent="0.25">
       <c r="B24" s="2" t="s">
         <v>12</v>
       </c>
       <c r="C24" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D24" s="1" t="s">
+      <c r="D24" s="2" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="25" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="E24" s="2"/>
+    </row>
+    <row r="25" spans="2:5" ht="30" x14ac:dyDescent="0.25">
       <c r="B25" s="2" t="s">
         <v>13</v>
       </c>
       <c r="C25" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="D25" s="1" t="s">
+      <c r="D25" s="2" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="26" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="E25" s="2"/>
+    </row>
+    <row r="26" spans="2:5" ht="30" x14ac:dyDescent="0.25">
       <c r="B26" s="2" t="s">
         <v>14</v>
       </c>
       <c r="C26" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="D26" s="1" t="s">
+      <c r="D26" s="2" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="27" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="E26" s="2"/>
+    </row>
+    <row r="27" spans="2:5" ht="30" x14ac:dyDescent="0.25">
       <c r="B27" s="2" t="s">
         <v>23</v>
       </c>
       <c r="C27" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="D27" s="1" t="s">
+      <c r="D27" s="2" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="28" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="E27" s="2"/>
+    </row>
+    <row r="28" spans="2:5" ht="30" x14ac:dyDescent="0.25">
       <c r="B28" s="2" t="s">
         <v>26</v>
       </c>
       <c r="C28" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D28" s="1" t="s">
+      <c r="D28" s="2" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="29" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="E28" s="2"/>
+    </row>
+    <row r="29" spans="2:5" ht="30" x14ac:dyDescent="0.25">
       <c r="B29" s="2" t="s">
         <v>27</v>
       </c>
       <c r="C29" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="D29" s="1" t="s">
+      <c r="D29" s="2" t="s">
         <v>31</v>
       </c>
+      <c r="E29" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>